<commit_message>
Update Nalco data (2026-02-23 05:13:05 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F200"/>
+  <dimension ref="A1:F201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1381,23 +1381,23 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2041,23 +2041,23 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3841,23 +3841,23 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E114" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3871,23 +3871,23 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3931,23 +3931,23 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4081,23 +4081,23 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4321,23 +4321,23 @@
         </is>
       </c>
       <c r="D130" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4411,23 +4411,23 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4561,23 +4561,23 @@
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4801,23 +4801,23 @@
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5701,23 +5701,23 @@
         </is>
       </c>
       <c r="D176" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E176" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F176" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5821,23 +5821,23 @@
         </is>
       </c>
       <c r="D180" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E180" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F180" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6031,23 +6031,23 @@
         </is>
       </c>
       <c r="D187" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E187" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F187" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6211,23 +6211,23 @@
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E193" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F193" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6429,6 +6429,36 @@
         </is>
       </c>
       <c r="F200" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="1" t="inlineStr">
+        <is>
+          <t>07-08-2025</t>
+        </is>
+      </c>
+      <c r="B201" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C201" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="n">
+        <v>268.25</v>
+      </c>
+      <c r="E201" s="1" t="inlineStr">
+        <is>
+          <t>07-08-2025</t>
+        </is>
+      </c>
+      <c r="F201" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -6635,6 +6665,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F198" r:id="rId197"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId200"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-02-24 05:07:39 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F201"/>
+  <dimension ref="A1:F202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1141,23 +1141,23 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1411,23 +1411,23 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2071,23 +2071,23 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3871,23 +3871,23 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3901,23 +3901,23 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3961,23 +3961,23 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4111,23 +4111,23 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4351,23 +4351,23 @@
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4441,23 +4441,23 @@
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4591,23 +4591,23 @@
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4861,23 +4861,23 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5731,23 +5731,23 @@
         </is>
       </c>
       <c r="D177" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E177" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F177" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5851,23 +5851,23 @@
         </is>
       </c>
       <c r="D181" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E181" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F181" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6061,23 +6061,23 @@
         </is>
       </c>
       <c r="D188" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E188" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F188" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6241,23 +6241,23 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E194" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F194" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6459,6 +6459,36 @@
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="1" t="inlineStr">
+        <is>
+          <t>07-08-2025</t>
+        </is>
+      </c>
+      <c r="B202" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C202" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="n">
+        <v>268.25</v>
+      </c>
+      <c r="E202" s="1" t="inlineStr">
+        <is>
+          <t>07-08-2025</t>
+        </is>
+      </c>
+      <c r="F202" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -6666,6 +6696,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F200" r:id="rId199"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F202" r:id="rId201"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-02-26 05:06:56 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F366"/>
+  <dimension ref="A1:F367"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1201,23 +1201,23 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2131,23 +2131,23 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3931,23 +3931,23 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3961,23 +3961,23 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4021,23 +4021,23 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4171,23 +4171,23 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4411,23 +4411,23 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4501,23 +4501,23 @@
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4651,23 +4651,23 @@
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4891,23 +4891,23 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4921,23 +4921,23 @@
         </is>
       </c>
       <c r="D150" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5311,23 +5311,23 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5791,23 +5791,23 @@
         </is>
       </c>
       <c r="D179" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E179" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F179" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5911,23 +5911,23 @@
         </is>
       </c>
       <c r="D183" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E183" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F183" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6121,23 +6121,23 @@
         </is>
       </c>
       <c r="D190" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E190" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6301,23 +6301,23 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E196" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F196" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11409,6 +11409,36 @@
         </is>
       </c>
       <c r="F366" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B367" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C367" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D367" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E367" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F367" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -11781,6 +11811,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F364" r:id="rId363"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F365" r:id="rId364"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F366" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F367" r:id="rId366"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-02-27 04:59:12 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F367"/>
+  <dimension ref="A1:F368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1351,23 +1351,23 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1501,23 +1501,23 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2161,23 +2161,23 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3961,23 +3961,23 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -3991,23 +3991,23 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4051,23 +4051,23 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4201,23 +4201,23 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4441,23 +4441,23 @@
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4531,23 +4531,23 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4681,23 +4681,23 @@
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4921,23 +4921,23 @@
         </is>
       </c>
       <c r="D150" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5341,23 +5341,23 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5821,23 +5821,23 @@
         </is>
       </c>
       <c r="D180" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E180" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F180" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5941,23 +5941,23 @@
         </is>
       </c>
       <c r="D184" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E184" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F184" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6151,23 +6151,23 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E191" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6571,23 +6571,23 @@
         </is>
       </c>
       <c r="D205" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E205" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F205" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11439,6 +11439,36 @@
         </is>
       </c>
       <c r="F367" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B368" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C368" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D368" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E368" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F368" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -11812,6 +11842,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F365" r:id="rId364"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F366" r:id="rId365"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F367" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F368" r:id="rId367"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-02-28 04:39:21 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F368"/>
+  <dimension ref="A1:F369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1381,23 +1381,23 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1531,23 +1531,23 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2191,23 +2191,23 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -3991,23 +3991,23 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4021,23 +4021,23 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4081,23 +4081,23 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4231,23 +4231,23 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4471,23 +4471,23 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4561,23 +4561,23 @@
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4711,23 +4711,23 @@
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5281,23 +5281,23 @@
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5371,23 +5371,23 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5851,23 +5851,23 @@
         </is>
       </c>
       <c r="D181" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E181" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F181" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5971,23 +5971,23 @@
         </is>
       </c>
       <c r="D185" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E185" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F185" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6181,23 +6181,23 @@
         </is>
       </c>
       <c r="D192" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E192" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F192" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6601,23 +6601,23 @@
         </is>
       </c>
       <c r="D206" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E206" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F206" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11469,6 +11469,36 @@
         </is>
       </c>
       <c r="F368" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B369" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C369" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D369" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E369" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F369" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -11843,6 +11873,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F366" r:id="rId365"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F367" r:id="rId366"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F368" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F369" r:id="rId368"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-01 05:06:33 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F369"/>
+  <dimension ref="A1:F370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1291,23 +1291,23 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1411,23 +1411,23 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1561,23 +1561,23 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2221,23 +2221,23 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4021,23 +4021,23 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4051,23 +4051,23 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4111,23 +4111,23 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4261,23 +4261,23 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4501,23 +4501,23 @@
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4591,23 +4591,23 @@
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4741,23 +4741,23 @@
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5311,23 +5311,23 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5401,23 +5401,23 @@
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5881,23 +5881,23 @@
         </is>
       </c>
       <c r="D182" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E182" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F182" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6001,23 +6001,23 @@
         </is>
       </c>
       <c r="D186" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E186" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F186" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6211,23 +6211,23 @@
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E193" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F193" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6391,23 +6391,23 @@
         </is>
       </c>
       <c r="D199" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E199" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6631,23 +6631,23 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E207" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F207" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11499,6 +11499,36 @@
         </is>
       </c>
       <c r="F369" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B370" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C370" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D370" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E370" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F370" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -11874,6 +11904,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F367" r:id="rId366"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F368" r:id="rId367"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F369" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F370" r:id="rId369"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-02 05:02:20 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F370"/>
+  <dimension ref="A1:F371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1441,23 +1441,23 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1591,23 +1591,23 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2251,23 +2251,23 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4051,23 +4051,23 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4081,23 +4081,23 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4141,23 +4141,23 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4291,23 +4291,23 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4531,23 +4531,23 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4621,23 +4621,23 @@
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4771,23 +4771,23 @@
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5341,23 +5341,23 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5431,23 +5431,23 @@
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5911,23 +5911,23 @@
         </is>
       </c>
       <c r="D183" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E183" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F183" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6031,23 +6031,23 @@
         </is>
       </c>
       <c r="D187" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E187" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F187" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6241,23 +6241,23 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E194" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F194" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6421,23 +6421,23 @@
         </is>
       </c>
       <c r="D200" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E200" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F200" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6661,23 +6661,23 @@
         </is>
       </c>
       <c r="D208" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E208" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F208" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11529,6 +11529,36 @@
         </is>
       </c>
       <c r="F370" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B371" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C371" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D371" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E371" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F371" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -11905,6 +11935,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F368" r:id="rId367"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F369" r:id="rId368"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F370" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F371" r:id="rId370"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-03 04:59:46 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F371"/>
+  <dimension ref="A1:F372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,37 +467,37 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
+          <t>02-03-2026</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>339.45</v>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
           <t>01-03-2026</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>320.45</v>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>01-02-2026</t>
-        </is>
-      </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -511,23 +511,23 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1351,23 +1351,23 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1621,23 +1621,23 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2281,23 +2281,23 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4081,23 +4081,23 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4111,23 +4111,23 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4171,23 +4171,23 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4321,23 +4321,23 @@
         </is>
       </c>
       <c r="D130" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4561,23 +4561,23 @@
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4651,23 +4651,23 @@
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4801,23 +4801,23 @@
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5371,23 +5371,23 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5461,23 +5461,23 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5941,23 +5941,23 @@
         </is>
       </c>
       <c r="D184" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E184" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F184" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6061,23 +6061,23 @@
         </is>
       </c>
       <c r="D188" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E188" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F188" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6271,23 +6271,23 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E195" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F195" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6451,23 +6451,23 @@
         </is>
       </c>
       <c r="D201" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6691,23 +6691,23 @@
         </is>
       </c>
       <c r="D209" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E209" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F209" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11559,6 +11559,36 @@
         </is>
       </c>
       <c r="F371" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B372" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C372" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D372" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E372" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F372" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -11936,6 +11966,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F369" r:id="rId368"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F370" r:id="rId369"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F371" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F372" r:id="rId371"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-04 04:53:45 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F372"/>
+  <dimension ref="A1:F373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -541,23 +541,23 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1381,23 +1381,23 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1501,23 +1501,23 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1921,23 +1921,23 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2311,23 +2311,23 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4111,23 +4111,23 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4141,23 +4141,23 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4201,23 +4201,23 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4351,23 +4351,23 @@
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4591,23 +4591,23 @@
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4681,23 +4681,23 @@
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5401,23 +5401,23 @@
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5491,23 +5491,23 @@
         </is>
       </c>
       <c r="D169" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5971,23 +5971,23 @@
         </is>
       </c>
       <c r="D185" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E185" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F185" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6091,23 +6091,23 @@
         </is>
       </c>
       <c r="D189" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E189" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F189" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6301,23 +6301,23 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E196" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F196" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6481,23 +6481,23 @@
         </is>
       </c>
       <c r="D202" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F202" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6721,23 +6721,23 @@
         </is>
       </c>
       <c r="D210" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E210" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F210" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11589,6 +11589,36 @@
         </is>
       </c>
       <c r="F372" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B373" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C373" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D373" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E373" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F373" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -11967,6 +11997,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F370" r:id="rId369"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F371" r:id="rId370"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F372" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F373" r:id="rId372"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-05 04:58:50 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F373"/>
+  <dimension ref="A1:F374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -571,23 +571,23 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1411,23 +1411,23 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1531,23 +1531,23 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1951,23 +1951,23 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2341,23 +2341,23 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4141,23 +4141,23 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4171,23 +4171,23 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4231,23 +4231,23 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4381,23 +4381,23 @@
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4621,23 +4621,23 @@
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4711,23 +4711,23 @@
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4861,23 +4861,23 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5281,23 +5281,23 @@
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5431,23 +5431,23 @@
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5521,23 +5521,23 @@
         </is>
       </c>
       <c r="D170" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6001,23 +6001,23 @@
         </is>
       </c>
       <c r="D186" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E186" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F186" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6121,23 +6121,23 @@
         </is>
       </c>
       <c r="D190" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E190" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6511,23 +6511,23 @@
         </is>
       </c>
       <c r="D203" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E203" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F203" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6751,23 +6751,23 @@
         </is>
       </c>
       <c r="D211" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E211" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F211" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11619,6 +11619,36 @@
         </is>
       </c>
       <c r="F373" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B374" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C374" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E374" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F374" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -11998,6 +12028,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F371" r:id="rId370"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F372" r:id="rId371"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F373" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F374" r:id="rId373"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-06 04:54:55 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F374"/>
+  <dimension ref="A1:F375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1441,23 +1441,23 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1561,23 +1561,23 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1981,23 +1981,23 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2371,23 +2371,23 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4171,23 +4171,23 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4201,23 +4201,23 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4261,23 +4261,23 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4411,23 +4411,23 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4651,23 +4651,23 @@
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4741,23 +4741,23 @@
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4891,23 +4891,23 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5311,23 +5311,23 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5461,23 +5461,23 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5551,23 +5551,23 @@
         </is>
       </c>
       <c r="D171" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E171" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F171" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6031,23 +6031,23 @@
         </is>
       </c>
       <c r="D187" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E187" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F187" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6151,23 +6151,23 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E191" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6781,23 +6781,23 @@
         </is>
       </c>
       <c r="D212" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E212" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F212" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="374">
       <c r="A374" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B374" s="1" t="inlineStr">
@@ -11649,6 +11649,36 @@
         </is>
       </c>
       <c r="F374" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B375" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C375" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D375" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E375" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F375" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -12029,6 +12059,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F372" r:id="rId371"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F373" r:id="rId372"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F374" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F375" r:id="rId374"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-07 04:45:10 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F375"/>
+  <dimension ref="A1:F376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1591,23 +1591,23 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2011,23 +2011,23 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2401,23 +2401,23 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4201,23 +4201,23 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4231,23 +4231,23 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4291,23 +4291,23 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4441,23 +4441,23 @@
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4681,23 +4681,23 @@
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4771,23 +4771,23 @@
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4921,23 +4921,23 @@
         </is>
       </c>
       <c r="D150" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5341,23 +5341,23 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5491,23 +5491,23 @@
         </is>
       </c>
       <c r="D169" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5581,23 +5581,23 @@
         </is>
       </c>
       <c r="D172" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E172" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F172" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6061,23 +6061,23 @@
         </is>
       </c>
       <c r="D188" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E188" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F188" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6181,23 +6181,23 @@
         </is>
       </c>
       <c r="D192" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E192" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F192" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6391,23 +6391,23 @@
         </is>
       </c>
       <c r="D199" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E199" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6571,23 +6571,23 @@
         </is>
       </c>
       <c r="D205" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E205" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F205" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6811,23 +6811,23 @@
         </is>
       </c>
       <c r="D213" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E213" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F213" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="374">
       <c r="A374" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B374" s="1" t="inlineStr">
@@ -11657,7 +11657,7 @@
     <row r="375">
       <c r="A375" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B375" s="1" t="inlineStr">
@@ -11679,6 +11679,36 @@
         </is>
       </c>
       <c r="F375" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B376" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C376" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D376" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E376" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F376" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -12060,6 +12090,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F373" r:id="rId372"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F374" r:id="rId373"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F375" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F376" r:id="rId375"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-08 04:56:06 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F376"/>
+  <dimension ref="A1:F377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1501,23 +1501,23 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1621,23 +1621,23 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2041,23 +2041,23 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2431,23 +2431,23 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4231,23 +4231,23 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4261,23 +4261,23 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4321,23 +4321,23 @@
         </is>
       </c>
       <c r="D130" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4471,23 +4471,23 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4711,23 +4711,23 @@
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4801,23 +4801,23 @@
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5371,23 +5371,23 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5521,23 +5521,23 @@
         </is>
       </c>
       <c r="D170" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5611,23 +5611,23 @@
         </is>
       </c>
       <c r="D173" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E173" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F173" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6091,23 +6091,23 @@
         </is>
       </c>
       <c r="D189" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E189" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F189" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6211,23 +6211,23 @@
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E193" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F193" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6421,23 +6421,23 @@
         </is>
       </c>
       <c r="D200" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E200" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F200" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6601,23 +6601,23 @@
         </is>
       </c>
       <c r="D206" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E206" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F206" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6841,23 +6841,23 @@
         </is>
       </c>
       <c r="D214" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E214" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F214" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="374">
       <c r="A374" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B374" s="1" t="inlineStr">
@@ -11657,7 +11657,7 @@
     <row r="375">
       <c r="A375" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B375" s="1" t="inlineStr">
@@ -11687,7 +11687,7 @@
     <row r="376">
       <c r="A376" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B376" s="1" t="inlineStr">
@@ -11709,6 +11709,36 @@
         </is>
       </c>
       <c r="F376" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B377" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C377" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D377" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E377" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F377" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -12091,6 +12121,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F374" r:id="rId373"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F375" r:id="rId374"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F376" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F377" r:id="rId376"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-09 05:07:32 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F377"/>
+  <dimension ref="A1:F378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>07-03-2026</t>
+          <t>08-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1531,23 +1531,23 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2071,23 +2071,23 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2461,23 +2461,23 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4261,23 +4261,23 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4291,23 +4291,23 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4351,23 +4351,23 @@
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4501,23 +4501,23 @@
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4741,23 +4741,23 @@
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5401,23 +5401,23 @@
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5551,23 +5551,23 @@
         </is>
       </c>
       <c r="D171" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E171" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F171" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5641,23 +5641,23 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E174" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F174" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6121,23 +6121,23 @@
         </is>
       </c>
       <c r="D190" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E190" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6241,23 +6241,23 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E194" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F194" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6451,23 +6451,23 @@
         </is>
       </c>
       <c r="D201" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6631,23 +6631,23 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E207" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F207" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6871,23 +6871,23 @@
         </is>
       </c>
       <c r="D215" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E215" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F215" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="374">
       <c r="A374" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B374" s="1" t="inlineStr">
@@ -11657,7 +11657,7 @@
     <row r="375">
       <c r="A375" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B375" s="1" t="inlineStr">
@@ -11687,7 +11687,7 @@
     <row r="376">
       <c r="A376" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B376" s="1" t="inlineStr">
@@ -11717,7 +11717,7 @@
     <row r="377">
       <c r="A377" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B377" s="1" t="inlineStr">
@@ -11739,6 +11739,36 @@
         </is>
       </c>
       <c r="F377" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B378" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C378" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D378" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E378" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F378" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -12122,6 +12152,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F375" r:id="rId374"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F376" r:id="rId375"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F377" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F378" r:id="rId377"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-10 04:54:53 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F378"/>
+  <dimension ref="A1:F379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>08-03-2026</t>
+          <t>09-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>07-03-2026</t>
+          <t>08-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1561,23 +1561,23 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2101,23 +2101,23 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2491,23 +2491,23 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4291,23 +4291,23 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4321,23 +4321,23 @@
         </is>
       </c>
       <c r="D130" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4381,23 +4381,23 @@
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4531,23 +4531,23 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4771,23 +4771,23 @@
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4861,23 +4861,23 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5281,23 +5281,23 @@
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5431,23 +5431,23 @@
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5581,23 +5581,23 @@
         </is>
       </c>
       <c r="D172" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E172" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F172" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5671,23 +5671,23 @@
         </is>
       </c>
       <c r="D175" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E175" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F175" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6151,23 +6151,23 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E191" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6271,23 +6271,23 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E195" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F195" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6481,23 +6481,23 @@
         </is>
       </c>
       <c r="D202" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F202" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6661,23 +6661,23 @@
         </is>
       </c>
       <c r="D208" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E208" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F208" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6901,23 +6901,23 @@
         </is>
       </c>
       <c r="D216" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E216" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F216" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="374">
       <c r="A374" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B374" s="1" t="inlineStr">
@@ -11657,7 +11657,7 @@
     <row r="375">
       <c r="A375" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B375" s="1" t="inlineStr">
@@ -11687,7 +11687,7 @@
     <row r="376">
       <c r="A376" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B376" s="1" t="inlineStr">
@@ -11717,7 +11717,7 @@
     <row r="377">
       <c r="A377" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B377" s="1" t="inlineStr">
@@ -11747,7 +11747,7 @@
     <row r="378">
       <c r="A378" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B378" s="1" t="inlineStr">
@@ -11769,6 +11769,36 @@
         </is>
       </c>
       <c r="F378" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B379" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C379" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D379" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E379" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F379" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -12153,6 +12183,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F376" r:id="rId375"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F377" r:id="rId376"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F378" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F379" r:id="rId378"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-11 04:56:11 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F379"/>
+  <dimension ref="A1:F380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>09-03-2026</t>
+          <t>10-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>08-03-2026</t>
+          <t>09-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>07-03-2026</t>
+          <t>08-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -751,23 +751,23 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1591,23 +1591,23 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2131,23 +2131,23 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2521,23 +2521,23 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4321,23 +4321,23 @@
         </is>
       </c>
       <c r="D130" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4351,23 +4351,23 @@
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4411,23 +4411,23 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4561,23 +4561,23 @@
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4801,23 +4801,23 @@
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4891,23 +4891,23 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5281,23 +5281,23 @@
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5311,23 +5311,23 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5461,23 +5461,23 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5611,23 +5611,23 @@
         </is>
       </c>
       <c r="D173" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E173" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F173" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5701,23 +5701,23 @@
         </is>
       </c>
       <c r="D176" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E176" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F176" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6181,23 +6181,23 @@
         </is>
       </c>
       <c r="D192" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E192" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F192" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6301,23 +6301,23 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E196" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F196" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6511,23 +6511,23 @@
         </is>
       </c>
       <c r="D203" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E203" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F203" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6691,23 +6691,23 @@
         </is>
       </c>
       <c r="D209" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E209" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F209" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6931,23 +6931,23 @@
         </is>
       </c>
       <c r="D217" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E217" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F217" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="374">
       <c r="A374" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B374" s="1" t="inlineStr">
@@ -11657,7 +11657,7 @@
     <row r="375">
       <c r="A375" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B375" s="1" t="inlineStr">
@@ -11687,7 +11687,7 @@
     <row r="376">
       <c r="A376" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B376" s="1" t="inlineStr">
@@ -11717,7 +11717,7 @@
     <row r="377">
       <c r="A377" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B377" s="1" t="inlineStr">
@@ -11747,7 +11747,7 @@
     <row r="378">
       <c r="A378" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B378" s="1" t="inlineStr">
@@ -11777,7 +11777,7 @@
     <row r="379">
       <c r="A379" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B379" s="1" t="inlineStr">
@@ -11799,6 +11799,36 @@
         </is>
       </c>
       <c r="F379" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B380" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C380" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D380" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E380" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F380" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -12184,6 +12214,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F377" r:id="rId376"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F378" r:id="rId377"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F379" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F380" r:id="rId379"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-12 05:01:11 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F380"/>
+  <dimension ref="A1:F381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>10-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>09-03-2026</t>
+          <t>10-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>08-03-2026</t>
+          <t>09-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>07-03-2026</t>
+          <t>08-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1621,23 +1621,23 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2161,23 +2161,23 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2551,23 +2551,23 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4351,23 +4351,23 @@
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4381,23 +4381,23 @@
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4441,23 +4441,23 @@
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4591,23 +4591,23 @@
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4921,23 +4921,23 @@
         </is>
       </c>
       <c r="D150" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5311,23 +5311,23 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5341,23 +5341,23 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5491,23 +5491,23 @@
         </is>
       </c>
       <c r="D169" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5641,23 +5641,23 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E174" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F174" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5731,23 +5731,23 @@
         </is>
       </c>
       <c r="D177" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E177" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F177" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6211,23 +6211,23 @@
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E193" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F193" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6721,23 +6721,23 @@
         </is>
       </c>
       <c r="D210" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E210" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F210" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6961,23 +6961,23 @@
         </is>
       </c>
       <c r="D218" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E218" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F218" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="374">
       <c r="A374" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B374" s="1" t="inlineStr">
@@ -11657,7 +11657,7 @@
     <row r="375">
       <c r="A375" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B375" s="1" t="inlineStr">
@@ -11687,7 +11687,7 @@
     <row r="376">
       <c r="A376" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B376" s="1" t="inlineStr">
@@ -11717,7 +11717,7 @@
     <row r="377">
       <c r="A377" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B377" s="1" t="inlineStr">
@@ -11747,7 +11747,7 @@
     <row r="378">
       <c r="A378" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B378" s="1" t="inlineStr">
@@ -11777,7 +11777,7 @@
     <row r="379">
       <c r="A379" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B379" s="1" t="inlineStr">
@@ -11807,7 +11807,7 @@
     <row r="380">
       <c r="A380" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B380" s="1" t="inlineStr">
@@ -11829,6 +11829,36 @@
         </is>
       </c>
       <c r="F380" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B381" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C381" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D381" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E381" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F381" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -12215,6 +12245,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F378" r:id="rId377"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F379" r:id="rId378"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F380" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F381" r:id="rId380"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-13 04:58:19 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F381"/>
+  <dimension ref="A1:F382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>12-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>10-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>09-03-2026</t>
+          <t>10-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>08-03-2026</t>
+          <t>09-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>07-03-2026</t>
+          <t>08-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1921,23 +1921,23 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2191,23 +2191,23 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2581,23 +2581,23 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4381,23 +4381,23 @@
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4411,23 +4411,23 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4471,23 +4471,23 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4621,23 +4621,23 @@
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4861,23 +4861,23 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5341,23 +5341,23 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5371,23 +5371,23 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5521,23 +5521,23 @@
         </is>
       </c>
       <c r="D170" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5671,23 +5671,23 @@
         </is>
       </c>
       <c r="D175" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E175" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F175" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5761,23 +5761,23 @@
         </is>
       </c>
       <c r="D178" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E178" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F178" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6241,23 +6241,23 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E194" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F194" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6571,23 +6571,23 @@
         </is>
       </c>
       <c r="D205" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E205" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F205" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6751,23 +6751,23 @@
         </is>
       </c>
       <c r="D211" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E211" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F211" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -6991,23 +6991,23 @@
         </is>
       </c>
       <c r="D219" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E219" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F219" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="374">
       <c r="A374" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B374" s="1" t="inlineStr">
@@ -11657,7 +11657,7 @@
     <row r="375">
       <c r="A375" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B375" s="1" t="inlineStr">
@@ -11687,7 +11687,7 @@
     <row r="376">
       <c r="A376" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B376" s="1" t="inlineStr">
@@ -11717,7 +11717,7 @@
     <row r="377">
       <c r="A377" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B377" s="1" t="inlineStr">
@@ -11747,7 +11747,7 @@
     <row r="378">
       <c r="A378" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B378" s="1" t="inlineStr">
@@ -11777,7 +11777,7 @@
     <row r="379">
       <c r="A379" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B379" s="1" t="inlineStr">
@@ -11807,7 +11807,7 @@
     <row r="380">
       <c r="A380" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B380" s="1" t="inlineStr">
@@ -11837,7 +11837,7 @@
     <row r="381">
       <c r="A381" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B381" s="1" t="inlineStr">
@@ -11859,6 +11859,36 @@
         </is>
       </c>
       <c r="F381" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B382" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C382" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D382" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E382" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F382" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -12246,6 +12276,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F379" r:id="rId378"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F380" r:id="rId379"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F381" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F382" r:id="rId381"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-14 04:56:20 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F382"/>
+  <dimension ref="A1:F383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>12-03-2026</t>
+          <t>13-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>12-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>10-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>09-03-2026</t>
+          <t>10-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>08-03-2026</t>
+          <t>09-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>07-03-2026</t>
+          <t>08-03-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1951,23 +1951,23 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2221,23 +2221,23 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2611,23 +2611,23 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4411,23 +4411,23 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4441,23 +4441,23 @@
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4501,23 +4501,23 @@
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4651,23 +4651,23 @@
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4891,23 +4891,23 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5371,23 +5371,23 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5401,23 +5401,23 @@
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5551,23 +5551,23 @@
         </is>
       </c>
       <c r="D171" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E171" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F171" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5701,23 +5701,23 @@
         </is>
       </c>
       <c r="D176" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E176" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F176" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5791,23 +5791,23 @@
         </is>
       </c>
       <c r="D179" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E179" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F179" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6271,23 +6271,23 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E195" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F195" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6391,23 +6391,23 @@
         </is>
       </c>
       <c r="D199" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E199" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6601,23 +6601,23 @@
         </is>
       </c>
       <c r="D206" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E206" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F206" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6781,23 +6781,23 @@
         </is>
       </c>
       <c r="D212" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E212" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F212" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7021,23 +7021,23 @@
         </is>
       </c>
       <c r="D220" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E220" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F220" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="374">
       <c r="A374" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B374" s="1" t="inlineStr">
@@ -11657,7 +11657,7 @@
     <row r="375">
       <c r="A375" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B375" s="1" t="inlineStr">
@@ -11687,7 +11687,7 @@
     <row r="376">
       <c r="A376" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B376" s="1" t="inlineStr">
@@ -11717,7 +11717,7 @@
     <row r="377">
       <c r="A377" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B377" s="1" t="inlineStr">
@@ -11747,7 +11747,7 @@
     <row r="378">
       <c r="A378" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B378" s="1" t="inlineStr">
@@ -11777,7 +11777,7 @@
     <row r="379">
       <c r="A379" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B379" s="1" t="inlineStr">
@@ -11807,7 +11807,7 @@
     <row r="380">
       <c r="A380" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B380" s="1" t="inlineStr">
@@ -11837,7 +11837,7 @@
     <row r="381">
       <c r="A381" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B381" s="1" t="inlineStr">
@@ -11867,7 +11867,7 @@
     <row r="382">
       <c r="A382" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B382" s="1" t="inlineStr">
@@ -11889,6 +11889,36 @@
         </is>
       </c>
       <c r="F382" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B383" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C383" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D383" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E383" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F383" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -12277,6 +12307,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F380" r:id="rId379"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F381" r:id="rId380"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F382" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F383" r:id="rId382"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-15 05:16:40 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F383"/>
+  <dimension ref="A1:F384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>13-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>12-03-2026</t>
+          <t>13-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>12-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>10-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>09-03-2026</t>
+          <t>10-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>08-03-2026</t>
+          <t>09-03-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>07-03-2026</t>
+          <t>08-03-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1981,23 +1981,23 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2251,23 +2251,23 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2641,23 +2641,23 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4441,23 +4441,23 @@
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4471,23 +4471,23 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4531,23 +4531,23 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4681,23 +4681,23 @@
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4921,23 +4921,23 @@
         </is>
       </c>
       <c r="D150" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5401,23 +5401,23 @@
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5431,23 +5431,23 @@
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5581,23 +5581,23 @@
         </is>
       </c>
       <c r="D172" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E172" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F172" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5731,23 +5731,23 @@
         </is>
       </c>
       <c r="D177" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E177" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F177" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5821,23 +5821,23 @@
         </is>
       </c>
       <c r="D180" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E180" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F180" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6301,23 +6301,23 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E196" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F196" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6421,23 +6421,23 @@
         </is>
       </c>
       <c r="D200" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E200" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F200" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6631,23 +6631,23 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E207" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F207" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6811,23 +6811,23 @@
         </is>
       </c>
       <c r="D213" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E213" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F213" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7051,23 +7051,23 @@
         </is>
       </c>
       <c r="D221" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E221" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F221" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="374">
       <c r="A374" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B374" s="1" t="inlineStr">
@@ -11657,7 +11657,7 @@
     <row r="375">
       <c r="A375" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B375" s="1" t="inlineStr">
@@ -11687,7 +11687,7 @@
     <row r="376">
       <c r="A376" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B376" s="1" t="inlineStr">
@@ -11717,7 +11717,7 @@
     <row r="377">
       <c r="A377" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B377" s="1" t="inlineStr">
@@ -11747,7 +11747,7 @@
     <row r="378">
       <c r="A378" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B378" s="1" t="inlineStr">
@@ -11777,7 +11777,7 @@
     <row r="379">
       <c r="A379" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B379" s="1" t="inlineStr">
@@ -11807,7 +11807,7 @@
     <row r="380">
       <c r="A380" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B380" s="1" t="inlineStr">
@@ -11837,7 +11837,7 @@
     <row r="381">
       <c r="A381" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B381" s="1" t="inlineStr">
@@ -11867,7 +11867,7 @@
     <row r="382">
       <c r="A382" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B382" s="1" t="inlineStr">
@@ -11897,7 +11897,7 @@
     <row r="383">
       <c r="A383" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B383" s="1" t="inlineStr">
@@ -11919,6 +11919,36 @@
         </is>
       </c>
       <c r="F383" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B384" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C384" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D384" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E384" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F384" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -12308,6 +12338,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F381" r:id="rId380"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F382" r:id="rId381"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F383" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F384" r:id="rId383"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-16 05:27:50 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F384"/>
+  <dimension ref="A1:F385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>15-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>13-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>12-03-2026</t>
+          <t>13-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>12-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>10-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>09-03-2026</t>
+          <t>10-03-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>08-03-2026</t>
+          <t>09-03-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>07-03-2026</t>
+          <t>08-03-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2011,23 +2011,23 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2281,23 +2281,23 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2671,23 +2671,23 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4471,23 +4471,23 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4501,23 +4501,23 @@
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4561,23 +4561,23 @@
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4711,23 +4711,23 @@
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5431,23 +5431,23 @@
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5461,23 +5461,23 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5611,23 +5611,23 @@
         </is>
       </c>
       <c r="D173" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E173" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F173" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5761,23 +5761,23 @@
         </is>
       </c>
       <c r="D178" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E178" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F178" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5851,23 +5851,23 @@
         </is>
       </c>
       <c r="D181" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E181" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F181" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6451,23 +6451,23 @@
         </is>
       </c>
       <c r="D201" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6661,23 +6661,23 @@
         </is>
       </c>
       <c r="D208" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E208" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F208" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6841,23 +6841,23 @@
         </is>
       </c>
       <c r="D214" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E214" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F214" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7081,23 +7081,23 @@
         </is>
       </c>
       <c r="D222" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E222" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F222" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8417,7 +8417,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B267" s="1" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B268" s="1" t="inlineStr">
@@ -8477,7 +8477,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B269" s="1" t="inlineStr">
@@ -8507,7 +8507,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B270" s="1" t="inlineStr">
@@ -8537,7 +8537,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B271" s="1" t="inlineStr">
@@ -8567,7 +8567,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B272" s="1" t="inlineStr">
@@ -8597,7 +8597,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B273" s="1" t="inlineStr">
@@ -8627,7 +8627,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B274" s="1" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B275" s="1" t="inlineStr">
@@ -8687,7 +8687,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B276" s="1" t="inlineStr">
@@ -8717,7 +8717,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B277" s="1" t="inlineStr">
@@ -8747,7 +8747,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>11-06-2025</t>
+          <t>12-06-2025</t>
         </is>
       </c>
       <c r="B278" s="1" t="inlineStr">
@@ -8777,7 +8777,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>10-06-2025</t>
+          <t>11-06-2025</t>
         </is>
       </c>
       <c r="B279" s="1" t="inlineStr">
@@ -8807,7 +8807,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>09-06-2025</t>
+          <t>10-06-2025</t>
         </is>
       </c>
       <c r="B280" s="1" t="inlineStr">
@@ -8837,7 +8837,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>08-06-2025</t>
+          <t>09-06-2025</t>
         </is>
       </c>
       <c r="B281" s="1" t="inlineStr">
@@ -8867,7 +8867,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>07-06-2025</t>
+          <t>08-06-2025</t>
         </is>
       </c>
       <c r="B282" s="1" t="inlineStr">
@@ -8897,7 +8897,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>06-06-2025</t>
+          <t>07-06-2025</t>
         </is>
       </c>
       <c r="B283" s="1" t="inlineStr">
@@ -8927,7 +8927,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>05-06-2025</t>
+          <t>06-06-2025</t>
         </is>
       </c>
       <c r="B284" s="1" t="inlineStr">
@@ -8957,7 +8957,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>04-06-2025</t>
+          <t>05-06-2025</t>
         </is>
       </c>
       <c r="B285" s="1" t="inlineStr">
@@ -8987,7 +8987,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>03-06-2025</t>
+          <t>04-06-2025</t>
         </is>
       </c>
       <c r="B286" s="1" t="inlineStr">
@@ -9017,7 +9017,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>02-06-2025</t>
+          <t>03-06-2025</t>
         </is>
       </c>
       <c r="B287" s="1" t="inlineStr">
@@ -9047,7 +9047,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>02-06-2025</t>
         </is>
       </c>
       <c r="B288" s="1" t="inlineStr">
@@ -9077,7 +9077,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>31-05-2025</t>
+          <t>01-06-2025</t>
         </is>
       </c>
       <c r="B289" s="1" t="inlineStr">
@@ -9107,7 +9107,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>30-05-2025</t>
+          <t>31-05-2025</t>
         </is>
       </c>
       <c r="B290" s="1" t="inlineStr">
@@ -9137,7 +9137,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>29-05-2025</t>
+          <t>30-05-2025</t>
         </is>
       </c>
       <c r="B291" s="1" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>28-05-2025</t>
+          <t>29-05-2025</t>
         </is>
       </c>
       <c r="B292" s="1" t="inlineStr">
@@ -9197,7 +9197,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>27-05-2025</t>
+          <t>28-05-2025</t>
         </is>
       </c>
       <c r="B293" s="1" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>26-05-2025</t>
+          <t>27-05-2025</t>
         </is>
       </c>
       <c r="B294" s="1" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>25-05-2025</t>
+          <t>26-05-2025</t>
         </is>
       </c>
       <c r="B295" s="1" t="inlineStr">
@@ -9287,7 +9287,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>24-05-2025</t>
+          <t>25-05-2025</t>
         </is>
       </c>
       <c r="B296" s="1" t="inlineStr">
@@ -9317,7 +9317,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>23-05-2025</t>
+          <t>24-05-2025</t>
         </is>
       </c>
       <c r="B297" s="1" t="inlineStr">
@@ -9347,7 +9347,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>22-05-2025</t>
+          <t>23-05-2025</t>
         </is>
       </c>
       <c r="B298" s="1" t="inlineStr">
@@ -9377,7 +9377,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>21-05-2025</t>
+          <t>22-05-2025</t>
         </is>
       </c>
       <c r="B299" s="1" t="inlineStr">
@@ -9407,7 +9407,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>20-05-2025</t>
+          <t>21-05-2025</t>
         </is>
       </c>
       <c r="B300" s="1" t="inlineStr">
@@ -9437,7 +9437,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>19-05-2025</t>
+          <t>20-05-2025</t>
         </is>
       </c>
       <c r="B301" s="1" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>18-05-2025</t>
+          <t>19-05-2025</t>
         </is>
       </c>
       <c r="B302" s="1" t="inlineStr">
@@ -9497,7 +9497,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>17-05-2025</t>
+          <t>18-05-2025</t>
         </is>
       </c>
       <c r="B303" s="1" t="inlineStr">
@@ -9527,7 +9527,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>16-05-2025</t>
+          <t>17-05-2025</t>
         </is>
       </c>
       <c r="B304" s="1" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>15-05-2025</t>
+          <t>16-05-2025</t>
         </is>
       </c>
       <c r="B305" s="1" t="inlineStr">
@@ -9587,7 +9587,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>14-05-2025</t>
+          <t>15-05-2025</t>
         </is>
       </c>
       <c r="B306" s="1" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>14-05-2025</t>
         </is>
       </c>
       <c r="B307" s="1" t="inlineStr">
@@ -9647,7 +9647,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>12-05-2025</t>
+          <t>13-05-2025</t>
         </is>
       </c>
       <c r="B308" s="1" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>11-05-2025</t>
+          <t>12-05-2025</t>
         </is>
       </c>
       <c r="B309" s="1" t="inlineStr">
@@ -9707,7 +9707,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>10-05-2025</t>
+          <t>11-05-2025</t>
         </is>
       </c>
       <c r="B310" s="1" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>09-05-2025</t>
+          <t>10-05-2025</t>
         </is>
       </c>
       <c r="B311" s="1" t="inlineStr">
@@ -9767,7 +9767,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>08-05-2025</t>
+          <t>09-05-2025</t>
         </is>
       </c>
       <c r="B312" s="1" t="inlineStr">
@@ -9797,7 +9797,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>07-05-2025</t>
+          <t>08-05-2025</t>
         </is>
       </c>
       <c r="B313" s="1" t="inlineStr">
@@ -9827,7 +9827,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>06-05-2025</t>
+          <t>07-05-2025</t>
         </is>
       </c>
       <c r="B314" s="1" t="inlineStr">
@@ -9857,7 +9857,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>05-05-2025</t>
+          <t>06-05-2025</t>
         </is>
       </c>
       <c r="B315" s="1" t="inlineStr">
@@ -9887,7 +9887,7 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>04-05-2025</t>
+          <t>05-05-2025</t>
         </is>
       </c>
       <c r="B316" s="1" t="inlineStr">
@@ -9917,7 +9917,7 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>03-05-2025</t>
+          <t>04-05-2025</t>
         </is>
       </c>
       <c r="B317" s="1" t="inlineStr">
@@ -9947,7 +9947,7 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>02-05-2025</t>
+          <t>03-05-2025</t>
         </is>
       </c>
       <c r="B318" s="1" t="inlineStr">
@@ -9977,7 +9977,7 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>02-05-2025</t>
         </is>
       </c>
       <c r="B319" s="1" t="inlineStr">
@@ -10007,7 +10007,7 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>30-04-2025</t>
+          <t>01-05-2025</t>
         </is>
       </c>
       <c r="B320" s="1" t="inlineStr">
@@ -10037,7 +10037,7 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>29-04-2025</t>
+          <t>30-04-2025</t>
         </is>
       </c>
       <c r="B321" s="1" t="inlineStr">
@@ -10067,7 +10067,7 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>28-04-2025</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="B322" s="1" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>27-04-2025</t>
+          <t>28-04-2025</t>
         </is>
       </c>
       <c r="B323" s="1" t="inlineStr">
@@ -10127,7 +10127,7 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>26-04-2025</t>
+          <t>27-04-2025</t>
         </is>
       </c>
       <c r="B324" s="1" t="inlineStr">
@@ -10157,7 +10157,7 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>25-04-2025</t>
+          <t>26-04-2025</t>
         </is>
       </c>
       <c r="B325" s="1" t="inlineStr">
@@ -10187,7 +10187,7 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>24-04-2025</t>
+          <t>25-04-2025</t>
         </is>
       </c>
       <c r="B326" s="1" t="inlineStr">
@@ -10217,7 +10217,7 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>23-04-2025</t>
+          <t>24-04-2025</t>
         </is>
       </c>
       <c r="B327" s="1" t="inlineStr">
@@ -10247,7 +10247,7 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>22-04-2025</t>
+          <t>23-04-2025</t>
         </is>
       </c>
       <c r="B328" s="1" t="inlineStr">
@@ -10277,7 +10277,7 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>21-04-2025</t>
+          <t>22-04-2025</t>
         </is>
       </c>
       <c r="B329" s="1" t="inlineStr">
@@ -10307,7 +10307,7 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>20-04-2025</t>
+          <t>21-04-2025</t>
         </is>
       </c>
       <c r="B330" s="1" t="inlineStr">
@@ -10337,7 +10337,7 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>19-04-2025</t>
+          <t>20-04-2025</t>
         </is>
       </c>
       <c r="B331" s="1" t="inlineStr">
@@ -10367,7 +10367,7 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>18-04-2025</t>
+          <t>19-04-2025</t>
         </is>
       </c>
       <c r="B332" s="1" t="inlineStr">
@@ -10397,7 +10397,7 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>17-04-2025</t>
+          <t>18-04-2025</t>
         </is>
       </c>
       <c r="B333" s="1" t="inlineStr">
@@ -10427,7 +10427,7 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>17-04-2025</t>
         </is>
       </c>
       <c r="B334" s="1" t="inlineStr">
@@ -10457,7 +10457,7 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>15-04-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="B335" s="1" t="inlineStr">
@@ -10487,7 +10487,7 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>14-04-2025</t>
+          <t>15-04-2025</t>
         </is>
       </c>
       <c r="B336" s="1" t="inlineStr">
@@ -10517,7 +10517,7 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>13-04-2025</t>
+          <t>14-04-2025</t>
         </is>
       </c>
       <c r="B337" s="1" t="inlineStr">
@@ -10547,7 +10547,7 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>12-04-2025</t>
+          <t>13-04-2025</t>
         </is>
       </c>
       <c r="B338" s="1" t="inlineStr">
@@ -10577,7 +10577,7 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>11-04-2025</t>
+          <t>12-04-2025</t>
         </is>
       </c>
       <c r="B339" s="1" t="inlineStr">
@@ -10607,7 +10607,7 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>10-04-2025</t>
+          <t>11-04-2025</t>
         </is>
       </c>
       <c r="B340" s="1" t="inlineStr">
@@ -10637,7 +10637,7 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>09-04-2025</t>
+          <t>10-04-2025</t>
         </is>
       </c>
       <c r="B341" s="1" t="inlineStr">
@@ -10667,7 +10667,7 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>08-04-2025</t>
+          <t>09-04-2025</t>
         </is>
       </c>
       <c r="B342" s="1" t="inlineStr">
@@ -10697,7 +10697,7 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>07-04-2025</t>
+          <t>08-04-2025</t>
         </is>
       </c>
       <c r="B343" s="1" t="inlineStr">
@@ -10727,7 +10727,7 @@
     <row r="344">
       <c r="A344" s="1" t="inlineStr">
         <is>
-          <t>06-04-2025</t>
+          <t>07-04-2025</t>
         </is>
       </c>
       <c r="B344" s="1" t="inlineStr">
@@ -10757,7 +10757,7 @@
     <row r="345">
       <c r="A345" s="1" t="inlineStr">
         <is>
-          <t>05-04-2025</t>
+          <t>06-04-2025</t>
         </is>
       </c>
       <c r="B345" s="1" t="inlineStr">
@@ -10787,7 +10787,7 @@
     <row r="346">
       <c r="A346" s="1" t="inlineStr">
         <is>
-          <t>04-04-2025</t>
+          <t>05-04-2025</t>
         </is>
       </c>
       <c r="B346" s="1" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="347">
       <c r="A347" s="1" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
+          <t>04-04-2025</t>
         </is>
       </c>
       <c r="B347" s="1" t="inlineStr">
@@ -10847,7 +10847,7 @@
     <row r="348">
       <c r="A348" s="1" t="inlineStr">
         <is>
-          <t>02-04-2025</t>
+          <t>03-04-2025</t>
         </is>
       </c>
       <c r="B348" s="1" t="inlineStr">
@@ -10877,7 +10877,7 @@
     <row r="349">
       <c r="A349" s="1" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>02-04-2025</t>
         </is>
       </c>
       <c r="B349" s="1" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="350">
       <c r="A350" s="1" t="inlineStr">
         <is>
-          <t>31-03-2025</t>
+          <t>01-04-2025</t>
         </is>
       </c>
       <c r="B350" s="1" t="inlineStr">
@@ -10937,7 +10937,7 @@
     <row r="351">
       <c r="A351" s="1" t="inlineStr">
         <is>
-          <t>30-03-2025</t>
+          <t>31-03-2025</t>
         </is>
       </c>
       <c r="B351" s="1" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="352">
       <c r="A352" s="1" t="inlineStr">
         <is>
-          <t>29-03-2025</t>
+          <t>30-03-2025</t>
         </is>
       </c>
       <c r="B352" s="1" t="inlineStr">
@@ -10997,7 +10997,7 @@
     <row r="353">
       <c r="A353" s="1" t="inlineStr">
         <is>
-          <t>28-03-2025</t>
+          <t>29-03-2025</t>
         </is>
       </c>
       <c r="B353" s="1" t="inlineStr">
@@ -11027,7 +11027,7 @@
     <row r="354">
       <c r="A354" s="1" t="inlineStr">
         <is>
-          <t>27-03-2025</t>
+          <t>28-03-2025</t>
         </is>
       </c>
       <c r="B354" s="1" t="inlineStr">
@@ -11057,7 +11057,7 @@
     <row r="355">
       <c r="A355" s="1" t="inlineStr">
         <is>
-          <t>26-03-2025</t>
+          <t>27-03-2025</t>
         </is>
       </c>
       <c r="B355" s="1" t="inlineStr">
@@ -11087,7 +11087,7 @@
     <row r="356">
       <c r="A356" s="1" t="inlineStr">
         <is>
-          <t>25-03-2025</t>
+          <t>26-03-2025</t>
         </is>
       </c>
       <c r="B356" s="1" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="357">
       <c r="A357" s="1" t="inlineStr">
         <is>
-          <t>24-03-2025</t>
+          <t>25-03-2025</t>
         </is>
       </c>
       <c r="B357" s="1" t="inlineStr">
@@ -11147,7 +11147,7 @@
     <row r="358">
       <c r="A358" s="1" t="inlineStr">
         <is>
-          <t>23-03-2025</t>
+          <t>24-03-2025</t>
         </is>
       </c>
       <c r="B358" s="1" t="inlineStr">
@@ -11177,7 +11177,7 @@
     <row r="359">
       <c r="A359" s="1" t="inlineStr">
         <is>
-          <t>22-03-2025</t>
+          <t>23-03-2025</t>
         </is>
       </c>
       <c r="B359" s="1" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="360">
       <c r="A360" s="1" t="inlineStr">
         <is>
-          <t>21-03-2025</t>
+          <t>22-03-2025</t>
         </is>
       </c>
       <c r="B360" s="1" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="361">
       <c r="A361" s="1" t="inlineStr">
         <is>
-          <t>20-03-2025</t>
+          <t>21-03-2025</t>
         </is>
       </c>
       <c r="B361" s="1" t="inlineStr">
@@ -11267,7 +11267,7 @@
     <row r="362">
       <c r="A362" s="1" t="inlineStr">
         <is>
-          <t>19-03-2025</t>
+          <t>20-03-2025</t>
         </is>
       </c>
       <c r="B362" s="1" t="inlineStr">
@@ -11297,7 +11297,7 @@
     <row r="363">
       <c r="A363" s="1" t="inlineStr">
         <is>
-          <t>18-03-2025</t>
+          <t>19-03-2025</t>
         </is>
       </c>
       <c r="B363" s="1" t="inlineStr">
@@ -11327,7 +11327,7 @@
     <row r="364">
       <c r="A364" s="1" t="inlineStr">
         <is>
-          <t>17-03-2025</t>
+          <t>18-03-2025</t>
         </is>
       </c>
       <c r="B364" s="1" t="inlineStr">
@@ -11357,7 +11357,7 @@
     <row r="365">
       <c r="A365" s="1" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>17-03-2025</t>
         </is>
       </c>
       <c r="B365" s="1" t="inlineStr">
@@ -11387,7 +11387,7 @@
     <row r="366">
       <c r="A366" s="1" t="inlineStr">
         <is>
-          <t>15-03-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="B366" s="1" t="inlineStr">
@@ -11417,7 +11417,7 @@
     <row r="367">
       <c r="A367" s="1" t="inlineStr">
         <is>
-          <t>14-03-2025</t>
+          <t>15-03-2025</t>
         </is>
       </c>
       <c r="B367" s="1" t="inlineStr">
@@ -11447,7 +11447,7 @@
     <row r="368">
       <c r="A368" s="1" t="inlineStr">
         <is>
-          <t>13-03-2025</t>
+          <t>14-03-2025</t>
         </is>
       </c>
       <c r="B368" s="1" t="inlineStr">
@@ -11477,7 +11477,7 @@
     <row r="369">
       <c r="A369" s="1" t="inlineStr">
         <is>
-          <t>12-03-2025</t>
+          <t>13-03-2025</t>
         </is>
       </c>
       <c r="B369" s="1" t="inlineStr">
@@ -11507,7 +11507,7 @@
     <row r="370">
       <c r="A370" s="1" t="inlineStr">
         <is>
-          <t>11-03-2025</t>
+          <t>12-03-2025</t>
         </is>
       </c>
       <c r="B370" s="1" t="inlineStr">
@@ -11537,7 +11537,7 @@
     <row r="371">
       <c r="A371" s="1" t="inlineStr">
         <is>
-          <t>10-03-2025</t>
+          <t>11-03-2025</t>
         </is>
       </c>
       <c r="B371" s="1" t="inlineStr">
@@ -11567,7 +11567,7 @@
     <row r="372">
       <c r="A372" s="1" t="inlineStr">
         <is>
-          <t>09-03-2025</t>
+          <t>10-03-2025</t>
         </is>
       </c>
       <c r="B372" s="1" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="373">
       <c r="A373" s="1" t="inlineStr">
         <is>
-          <t>08-03-2025</t>
+          <t>09-03-2025</t>
         </is>
       </c>
       <c r="B373" s="1" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="374">
       <c r="A374" s="1" t="inlineStr">
         <is>
-          <t>07-03-2025</t>
+          <t>08-03-2025</t>
         </is>
       </c>
       <c r="B374" s="1" t="inlineStr">
@@ -11657,7 +11657,7 @@
     <row r="375">
       <c r="A375" s="1" t="inlineStr">
         <is>
-          <t>06-03-2025</t>
+          <t>07-03-2025</t>
         </is>
       </c>
       <c r="B375" s="1" t="inlineStr">
@@ -11687,7 +11687,7 @@
     <row r="376">
       <c r="A376" s="1" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>06-03-2025</t>
         </is>
       </c>
       <c r="B376" s="1" t="inlineStr">
@@ -11717,7 +11717,7 @@
     <row r="377">
       <c r="A377" s="1" t="inlineStr">
         <is>
-          <t>04-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="B377" s="1" t="inlineStr">
@@ -11747,7 +11747,7 @@
     <row r="378">
       <c r="A378" s="1" t="inlineStr">
         <is>
-          <t>03-03-2025</t>
+          <t>04-03-2025</t>
         </is>
       </c>
       <c r="B378" s="1" t="inlineStr">
@@ -11777,7 +11777,7 @@
     <row r="379">
       <c r="A379" s="1" t="inlineStr">
         <is>
-          <t>02-03-2025</t>
+          <t>03-03-2025</t>
         </is>
       </c>
       <c r="B379" s="1" t="inlineStr">
@@ -11807,7 +11807,7 @@
     <row r="380">
       <c r="A380" s="1" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>02-03-2025</t>
         </is>
       </c>
       <c r="B380" s="1" t="inlineStr">
@@ -11837,7 +11837,7 @@
     <row r="381">
       <c r="A381" s="1" t="inlineStr">
         <is>
-          <t>28-02-2025</t>
+          <t>01-03-2025</t>
         </is>
       </c>
       <c r="B381" s="1" t="inlineStr">
@@ -11867,7 +11867,7 @@
     <row r="382">
       <c r="A382" s="1" t="inlineStr">
         <is>
-          <t>27-02-2025</t>
+          <t>28-02-2025</t>
         </is>
       </c>
       <c r="B382" s="1" t="inlineStr">
@@ -11897,7 +11897,7 @@
     <row r="383">
       <c r="A383" s="1" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>27-02-2025</t>
         </is>
       </c>
       <c r="B383" s="1" t="inlineStr">
@@ -11927,7 +11927,7 @@
     <row r="384">
       <c r="A384" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="B384" s="1" t="inlineStr">
@@ -11949,6 +11949,36 @@
         </is>
       </c>
       <c r="F384" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="B385" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C385" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D385" s="2" t="n">
+        <v>323.05</v>
+      </c>
+      <c r="E385" s="1" t="inlineStr">
+        <is>
+          <t>25-02-2025</t>
+        </is>
+      </c>
+      <c r="F385" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
@@ -12339,6 +12369,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F382" r:id="rId381"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F383" r:id="rId382"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F384" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F385" r:id="rId384"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-03-17 05:07:59 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F385"/>
+  <dimension ref="A1:F386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>15-03-2026</t>
+          <t>16-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>15-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>13-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>12-03-2026</t>
+          <t>13-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>12-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>10-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>09-03-2026</t>
+          <t>10-03-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>08-03-2026</t>
+          <t>09-03-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>07-03-2026</t>
+          <t>08-03-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>320.45</v>
+        <v>339.45</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2041,23 +2041,23 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2311,23 +2311,23 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2701,23 +2701,23 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>296.05</v>
+        <v>320.05</v>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4501,23 +4501,23 @@
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4531,23 +4531,23 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4591,23 +4591,23 @@
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4741,23 +4741,23 @@
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5461,23 +5461,23 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5491,23 +5491,23 @@
         </is>
       </c>
       <c r="D169" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5641,23 +5641,23 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E174" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F174" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5791,23 +5791,23 @@
         </is>
       </c>
       <c r="D179" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E179" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F179" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5881,23 +5881,23 @@
         </is>
       </c>
       <c r="D182" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E182" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F182" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6481,23 +6481,23 @@
         </is>
       </c>
       <c r="D202" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F202" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6691,23 +6691,23 @@
         </is>
       </c>
       <c r="D209" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E209" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F209" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6871,23 +6871,23 @@
         </is>
       </c>
       <c r="D215" s="2" t="n">
-        <v>268.25</v>
+        <v>269.45</v>
       </c>
       <c r="E215" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="F215" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7111,23 +7111,23 @@
         </is>
       </c>
       <c r="D223" s="2" t="n">
-        <v>323.05</v>
+        <v>268.25</v>
       </c>
       <c r="E223" s="1" t="inlineStr">
         <is>
-          <t>25-02-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="F223" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+  